<commit_message>
2-1 edits - especially shiny app on covariance
</commit_message>
<xml_diff>
--- a/docs/handouts/chapter_2_1_handout.xlsx
+++ b/docs/handouts/chapter_2_1_handout.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\craigaj\Documents\GitHub\timeseries\docs\handouts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\craigaj\Documents\GitHub\timeseries\handouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EB39D67-466F-4456-B1E3-D7D35B769971}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8EF04BB-FF43-4206-BE5B-7FA5C6F71AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>sum</t>
   </si>
@@ -49,6 +49,9 @@
   </si>
   <si>
     <t>Table 3: Computational Practice</t>
+  </si>
+  <si>
+    <t>(Compute the unbiased estimators, dividing by n-1)</t>
   </si>
 </sst>
 </file>
@@ -75,11 +78,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="9.6"/>
       <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <name val="Source Sans Pro"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="14"/>
@@ -165,63 +167,85 @@
     </border>
     <border>
       <left style="thin">
-        <color theme="1"/>
+        <color indexed="64"/>
       </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
-        <color theme="1"/>
+        <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
+      <bottom style="thin">
         <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -231,24 +255,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2269,11 +2275,11 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>310674</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>74803</xdr:rowOff>
+      <xdr:rowOff>81153</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="122982" cy="221214"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="30" name="TextBox 29">
@@ -2287,7 +2293,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="310674" y="4754753"/>
+              <a:off x="310674" y="4627753"/>
               <a:ext cx="122982" cy="221214"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2333,7 +2339,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="30" name="TextBox 29">
@@ -2347,7 +2353,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="310674" y="4754753"/>
+              <a:off x="310674" y="4627753"/>
               <a:ext cx="122982" cy="221214"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2395,11 +2401,11 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>74454</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>81153</xdr:rowOff>
+      <xdr:rowOff>87503</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="735073" cy="221214"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="32" name="TextBox 31">
@@ -2413,7 +2419,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="74454" y="4380103"/>
+              <a:off x="74454" y="4253103"/>
               <a:ext cx="735073" cy="221214"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2489,7 +2495,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="32" name="TextBox 31">
@@ -2503,7 +2509,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="74454" y="4380103"/>
+              <a:off x="74454" y="4253103"/>
               <a:ext cx="735073" cy="221214"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2869,44 +2875,44 @@
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.90625" style="10" customWidth="1"/>
-    <col min="2" max="2" width="12" style="10" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" style="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="11.1796875" style="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12" style="10" customWidth="1"/>
-    <col min="8" max="8" width="18.1796875" style="10" customWidth="1"/>
-    <col min="9" max="13" width="8.7265625" style="10"/>
-    <col min="14" max="14" width="9.6328125" style="10" customWidth="1"/>
-    <col min="15" max="16384" width="8.7265625" style="10"/>
+    <col min="1" max="1" width="11.90625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="12" style="8" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="11.1796875" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12" style="8" customWidth="1"/>
+    <col min="8" max="8" width="18.1796875" style="8" customWidth="1"/>
+    <col min="9" max="13" width="8.7265625" style="8"/>
+    <col min="14" max="14" width="9.6328125" style="8" customWidth="1"/>
+    <col min="15" max="16384" width="8.7265625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="48.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="8"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="12"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
     </row>
-    <row r="3" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -2917,22 +2923,22 @@
         <v>2.8</v>
       </c>
       <c r="D3" s="4">
-        <v>-1.9000000000000001</v>
+        <v>-1.9</v>
       </c>
       <c r="E3" s="4">
-        <v>3.6100000000000003</v>
+        <v>3.61</v>
       </c>
       <c r="F3" s="4">
-        <v>0.99999999999999978</v>
+        <v>1</v>
       </c>
       <c r="G3" s="4">
-        <v>0.99999999999999956</v>
+        <v>1</v>
       </c>
       <c r="H3" s="4">
-        <v>-1.8999999999999997</v>
+        <v>-1.9</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <v>2</v>
       </c>
@@ -2942,13 +2948,13 @@
       <c r="C4" s="4">
         <v>2.2000000000000002</v>
       </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
     </row>
-    <row r="5" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>3</v>
       </c>
@@ -2958,13 +2964,13 @@
       <c r="C5" s="4">
         <v>0.9</v>
       </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
     </row>
-    <row r="6" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>4</v>
       </c>
@@ -2974,13 +2980,13 @@
       <c r="C6" s="4">
         <v>2</v>
       </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
     </row>
-    <row r="7" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>5</v>
       </c>
@@ -2990,13 +2996,13 @@
       <c r="C7" s="4">
         <v>-1</v>
       </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
     </row>
-    <row r="8" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>6</v>
       </c>
@@ -3006,54 +3012,57 @@
       <c r="C8" s="4">
         <v>3.9</v>
       </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
     </row>
-    <row r="9" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="6">
         <v>-1.2</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="6">
         <v>10.8</v>
       </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="10"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F11" s="13"/>
+      <c r="F11" s="11"/>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="14"/>
-      <c r="B12" s="9"/>
+      <c r="A12" s="9"/>
+      <c r="B12" s="12"/>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="14"/>
-      <c r="B13" s="9"/>
+      <c r="A13" s="9"/>
+      <c r="B13" s="12"/>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="14"/>
-      <c r="B14" s="9"/>
+      <c r="A14" s="9"/>
+      <c r="B14" s="12"/>
+      <c r="D14" s="13" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="14"/>
-      <c r="B15" s="9"/>
+      <c r="A15" s="9"/>
+      <c r="B15" s="12"/>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="14"/>
-      <c r="B16" s="9"/>
+      <c r="A16" s="9"/>
+      <c r="B16" s="12"/>
     </row>
     <row r="17" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="14"/>
-      <c r="B17" s="9"/>
+      <c r="A17" s="9"/>
+      <c r="B17" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3066,6 +3075,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010070F75838E79B0E48B83E8E3F5479A3A2" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2b0c304636f8f537543cd13f583db9d4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xmlns:ns4="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f089f22c5ce4e61126931f7622145b2" ns3:_="" ns4:_="">
     <xsd:import namespace="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
@@ -3260,38 +3286,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDDC771-C014-4A48-9FCA-802C556EA1D0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
-    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3314,9 +3312,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDDC771-C014-4A48-9FCA-802C556EA1D0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
+    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
2-1 edits - reversed order of r and cov(x,y)
</commit_message>
<xml_diff>
--- a/docs/handouts/chapter_2_1_handout.xlsx
+++ b/docs/handouts/chapter_2_1_handout.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\craigaj\Documents\GitHub\timeseries\handouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8EF04BB-FF43-4206-BE5B-7FA5C6F71AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB7991F6-13C6-4C26-869C-CD2FAF360F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
+    <workbookView xWindow="3720" yWindow="3720" windowWidth="19200" windowHeight="11170" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
   </bookViews>
   <sheets>
     <sheet name="Workbook" sheetId="2" r:id="rId1"/>
@@ -1982,14 +1982,14 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>318294</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>60833</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="197042" cy="221214"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="25" name="TextBox 24">
@@ -2068,7 +2068,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="25" name="TextBox 24">
@@ -2127,14 +2127,14 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>303054</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>45593</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="202235" cy="232436"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="29" name="TextBox 28">
@@ -2213,7 +2213,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="29" name="TextBox 28">
@@ -2272,14 +2272,14 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>310674</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>81153</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="122982" cy="221214"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="30" name="TextBox 29">
@@ -2339,7 +2339,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="30" name="TextBox 29">
@@ -2398,14 +2398,14 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>74454</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>87503</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="735073" cy="221214"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="32" name="TextBox 31">
@@ -2495,7 +2495,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="32" name="TextBox 31">
@@ -3035,35 +3035,31 @@
       <c r="H9" s="10"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D11" s="13" t="s">
+        <v>4</v>
+      </c>
       <c r="F11" s="11"/>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9"/>
       <c r="B12" s="12"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="12"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="12"/>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9"/>
       <c r="B13" s="12"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="12"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="12"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="9"/>
-      <c r="B14" s="12"/>
-      <c r="D14" s="13" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="9"/>
-      <c r="B15" s="12"/>
-    </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="9"/>
-      <c r="B16" s="12"/>
-    </row>
-    <row r="17" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="9"/>
-      <c r="B17" s="12"/>
-    </row>
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -3075,23 +3071,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010070F75838E79B0E48B83E8E3F5479A3A2" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2b0c304636f8f537543cd13f583db9d4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xmlns:ns4="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f089f22c5ce4e61126931f7622145b2" ns3:_="" ns4:_="">
     <xsd:import namespace="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
@@ -3286,10 +3265,38 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDDC771-C014-4A48-9FCA-802C556EA1D0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
+    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3312,20 +3319,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDDC771-C014-4A48-9FCA-802C556EA1D0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
-    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>